<commit_message>
running larger dataset experiments on bigbird
</commit_message>
<xml_diff>
--- a/nl_sql_results/nltosql-nosubset-abstract-Native-fullschema-nlsqlmodel_gemini-2.0-flash-lite-001.xlsx
+++ b/nl_sql_results/nltosql-nosubset-abstract-Native-fullschema-nlsqlmodel_gemini-2.0-flash-lite-001.xlsx
@@ -425,48 +425,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I1"/>
+  <dimension ref="B1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Unnamed: 0</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>database</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>question_number</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>nl_sql_model</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>generated_query</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>gold_query</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>nl_sql_tokens</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>result_set_match</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>non_match_reason</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>nl_sql_prompt_tokens</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
completed bigbird subsetting and most nl-to-sql
</commit_message>
<xml_diff>
--- a/nl_sql_results/nltosql-nosubset-abstract-Native-fullschema-nlsqlmodel_gemini-2.0-flash-lite-001.xlsx
+++ b/nl_sql_results/nltosql-nosubset-abstract-Native-fullschema-nlsqlmodel_gemini-2.0-flash-lite-001.xlsx
@@ -425,58 +425,48 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:K1"/>
+  <dimension ref="B1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Unnamed: 0</t>
+          <t>database</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>database</t>
+          <t>question_number</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>question_number</t>
+          <t>nl_sql_model</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>nl_sql_model</t>
+          <t>generated_query</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>generated_query</t>
+          <t>gold_query</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>gold_query</t>
+          <t>nl_sql_tokens</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>nl_sql_tokens</t>
+          <t>result_set_match</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>result_set_match</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
           <t>non_match_reason</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>nl_sql_prompt_tokens</t>
         </is>
       </c>
     </row>

</xml_diff>